<commit_message>
update: tambah biodata & simpan hasil diagnosis
</commit_message>
<xml_diff>
--- a/public/data/Bissmilah lagi.xlsx
+++ b/public/data/Bissmilah lagi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SEMPRO\Dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0B6B75A-CEEF-4B5D-A78F-5AD24E79B75C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AD0C0A7-3BBB-49D5-8A56-A94B87D2FC69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{080C0004-ABD4-4DE1-A00D-E05849B55E82}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>Penyakit</t>
   </si>
@@ -69,18 +69,9 @@
     <t>Jamur/Ringworm</t>
   </si>
   <si>
-    <t>Penyakit kutu dan pinjal serta gejala alergi kulit yang menyerta</t>
-  </si>
-  <si>
     <t>FLUTD (Feline Lower Urinary Tract Diseases)</t>
   </si>
   <si>
-    <t>URI (upper respirstory infection) bakterial</t>
-  </si>
-  <si>
-    <t>Diare Spesifik</t>
-  </si>
-  <si>
     <t>Diare Non Spesifik</t>
   </si>
   <si>
@@ -148,6 +139,24 @@
   </si>
   <si>
     <t>Berikan pakan berkualitas dan dalam jumlah yang cukup; Sediakan air minum bersih serta kotak pasir yang selalu terjaga kebersihannya; Lakukan pemberian obat cacing secara rutin; Sesuaikan pola makan dengan kebutuhan kucing sebagai karnivora, dan kelola stres agar kucing tetap sehat</t>
+  </si>
+  <si>
+    <t>Penyakit kutu dan pinjal</t>
+  </si>
+  <si>
+    <t>Pilek Kronis</t>
+  </si>
+  <si>
+    <t>Abses</t>
+  </si>
+  <si>
+    <t>Bakteri</t>
+  </si>
+  <si>
+    <t>Penanganan dilakukan dengan membersihkan area yang terinfeksi, mengeluarkan nanah, serta pemberian obat sesuai anjuran dokter hewan</t>
+  </si>
+  <si>
+    <t>Pencegahan dilakukan dengan menghindari perkelahian antar kucing; Menjaga kebersihan lingkungan; Segera membersihkan luka agar tidak terjadi infeksi</t>
   </si>
 </sst>
 </file>
@@ -309,7 +318,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -321,6 +329,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -639,207 +650,207 @@
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.77734375" style="8" customWidth="1"/>
-    <col min="2" max="2" width="20.5546875" style="8" customWidth="1"/>
-    <col min="3" max="3" width="40.109375" style="8" customWidth="1"/>
-    <col min="4" max="4" width="33.5546875" style="8" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="8"/>
+    <col min="1" max="1" width="40.77734375" style="12" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" style="12" customWidth="1"/>
+    <col min="3" max="3" width="40.109375" style="12" customWidth="1"/>
+    <col min="4" max="4" width="33.5546875" style="12" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>16</v>
+      <c r="B3" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>16</v>
+      <c r="B4" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>16</v>
+      <c r="B5" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="76.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>17</v>
+      <c r="B6" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>17</v>
+      <c r="B7" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>17</v>
+      <c r="B8" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="140.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>17</v>
+      <c r="B9" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="162" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B11" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="156" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="109.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="202.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="140.4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:4" ht="78" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>19</v>
+        <v>37</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>38</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="140.4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>19</v>
+        <v>12</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>16</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revisi data dan validasi
</commit_message>
<xml_diff>
--- a/public/data/Bissmilah lagi.xlsx
+++ b/public/data/Bissmilah lagi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SEMPRO\Dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AD0C0A7-3BBB-49D5-8A56-A94B87D2FC69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910E6CA2-8AFC-4CBB-AE13-0D8F448D34C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{080C0004-ABD4-4DE1-A00D-E05849B55E82}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
   <si>
     <t>Penyakit</t>
   </si>
@@ -154,9 +154,6 @@
   </si>
   <si>
     <t>Penanganan dilakukan dengan membersihkan area yang terinfeksi, mengeluarkan nanah, serta pemberian obat sesuai anjuran dokter hewan</t>
-  </si>
-  <si>
-    <t>Pencegahan dilakukan dengan menghindari perkelahian antar kucing; Menjaga kebersihan lingkungan; Segera membersihkan luka agar tidak terjadi infeksi</t>
   </si>
 </sst>
 </file>
@@ -825,7 +822,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="78" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="140.4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>37</v>
       </c>
@@ -836,7 +833,7 @@
         <v>39</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="140.4" x14ac:dyDescent="0.3">

</xml_diff>